<commit_message>
Update configurations and Excel report
</commit_message>
<xml_diff>
--- a/excel/Hodiny_Cap.xlsx
+++ b/excel/Hodiny_Cap.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Zálohy" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Týden" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Týden 15" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,9 +18,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="HH:MM"/>
     <numFmt numFmtId="165" formatCode="DD.MM.YYYY"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -50,11 +52,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,9 +423,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B80:H80"/>
+  <dimension ref="A8:Z80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Test 3</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="Z8" s="3" t="n">
+        <v>46121</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Horčička Jan</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>111</v>
+      </c>
+      <c r="Z9" s="3" t="n">
+        <v>46121</v>
+      </c>
+    </row>
     <row r="80">
       <c r="B80" t="inlineStr">
         <is>
@@ -461,4 +490,81 @@
   <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A4:G80"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>NÁZEV PROJEKTU : Ardo</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Čáp Jakub</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Horčička Jan</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="D80" s="3" t="n">
+        <v>46119</v>
+      </c>
+      <c r="F80" s="3" t="n">
+        <v>46120</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Aktualizace nastavení a skriptů
</commit_message>
<xml_diff>
--- a/excel/Hodiny_Cap.xlsx
+++ b/excel/Hodiny_Cap.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="Zálohy" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Týden" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Týden 15" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Týden 16" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -52,12 +52,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,35 +422,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A8:Z80"/>
+  <dimension ref="B80:H80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Test 3</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="Z8" s="3" t="n">
-        <v>46121</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Horčička Jan</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>111</v>
-      </c>
-      <c r="Z9" s="3" t="n">
-        <v>46121</v>
-      </c>
-    </row>
     <row r="80">
       <c r="B80" t="inlineStr">
         <is>
@@ -504,64 +477,45 @@
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>NÁZEV PROJEKTU : Ardo</t>
+          <t>NÁZEV PROJEKTU : Essity</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>08:00</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Čáp Jakub</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>9</v>
+          <t>Horčička Jan</t>
+        </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Horčička Jan</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="n">
-        <v>9</v>
+          <t>Čáp Jakub</t>
+        </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="80">
-      <c r="D80" s="3" t="n">
-        <v>46119</v>
-      </c>
       <c r="F80" s="3" t="n">
-        <v>46120</v>
+        <v>46127</v>
       </c>
     </row>
   </sheetData>

</xml_diff>